<commit_message>
producing result for analizying building graphv2 approach
</commit_message>
<xml_diff>
--- a/Perturbation/resumo_geral_grafo_cooc.xlsx
+++ b/Perturbation/resumo_geral_grafo_cooc.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DOUTORADO\units\XAI4Spectra\Perturbation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4331ED2-B08A-4A5D-B416-9C1311E48D0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D43467FC-FB71-4759-AEAE-01FF84EB9C01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{7256B89D-309C-4A19-B59F-B8F5A08FEBDA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{7256B89D-309C-4A19-B59F-B8F5A08FEBDA}"/>
   </bookViews>
   <sheets>
     <sheet name="synthetic" sheetId="3" r:id="rId1"/>
@@ -841,9 +841,9 @@
   <dimension ref="A1:J10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.44140625" style="2" customWidth="1"/>
     <col min="2" max="2" width="12.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.5546875" style="2" customWidth="1"/>
     <col min="4" max="4" width="14.109375" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.44140625" style="2" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.33203125" style="2" bestFit="1" customWidth="1"/>

</xml_diff>